<commit_message>
Refine adoption and parser behavior
Co-authored-by: sandeepsankarankutty <212097473+sandeepsankarankutty@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sample_data/sample_metrics.xlsx
+++ b/sample_data/sample_metrics.xlsx
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -577,25 +577,30 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Total test cases / month</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Number of test cases generated</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Test case coverage %</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Automation candidates identified</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Review defects found in test cases</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Review time per test case</t>
         </is>
@@ -625,18 +630,21 @@
         <v>0.8</v>
       </c>
       <c r="G2" t="n">
+        <v>520</v>
+      </c>
+      <c r="H2" t="n">
         <v>390</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>96</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>265</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>4</v>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>0.03</v>
       </c>
     </row>
@@ -664,18 +672,21 @@
         <v>0.7</v>
       </c>
       <c r="G3" t="n">
+        <v>410</v>
+      </c>
+      <c r="H3" t="n">
         <v>280</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>94</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>171</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>3</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>0.03</v>
       </c>
     </row>

</xml_diff>